<commit_message>
Auto: 2026-10-01 scrape results
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Health_and_Wellness.xlsx
+++ b/results/auto_Cape_Town_Health_and_Wellness.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -573,9 +573,6 @@
       <c r="D5" t="s">
         <v>30</v>
       </c>
-      <c r="G5" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -590,9 +587,6 @@
       <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -607,9 +601,6 @@
       <c r="D7" t="s">
         <v>32</v>
       </c>
-      <c r="G7" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -624,9 +615,6 @@
       <c r="D8" t="s">
         <v>33</v>
       </c>
-      <c r="G8" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -641,9 +629,6 @@
       <c r="D9" t="s">
         <v>34</v>
       </c>
-      <c r="G9" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -658,9 +643,6 @@
       <c r="D10" t="s">
         <v>35</v>
       </c>
-      <c r="G10" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -674,9 +656,6 @@
       </c>
       <c r="D11" t="s">
         <v>36</v>
-      </c>
-      <c r="G11" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:7">

</xml_diff>